<commit_message>
function: clean gold set and scraper
</commit_message>
<xml_diff>
--- a/src/scraping/data/cold_start/tesco.xlsx
+++ b/src/scraping/data/cold_start/tesco.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kumo/programming/competitor_product_search/src/scraping/data/cold_start/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yuding.Duan\OneDrive - Ipsos\3. self_projects\competitor_product_search\src\scraping\data\cold_start\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32BBA85-59E0-474C-98D6-263AC5DCD7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74201E26-B69A-4231-98C0-B07962014AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9840" yWindow="22360" windowWidth="24280" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cold_start" sheetId="1" r:id="rId1"/>
@@ -38,11 +38,11 @@
   </si>
   <si>
     <t>https://www.tesco.com/groceries/en-GB/products/276797313</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/325502056</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/305728358</t>
@@ -52,11 +52,11 @@
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/330702828</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>discounted</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/330671337</t>
@@ -66,7 +66,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -80,10 +80,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF1F2937"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Carlito"/>
     </font>
     <font>
@@ -176,28 +172,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="超链接" xfId="2" builtinId="8"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -408,13 +402,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="22" customHeight="1">
+    <row r="1" spans="1:2" ht="22.05" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -422,56 +416,56 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="22" customHeight="1">
+    <row r="2" spans="1:2" ht="22.05" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="22" customHeight="1">
+    <row r="3" spans="1:2" ht="22.05" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="22" customHeight="1">
+    <row r="4" spans="1:2" ht="22.05" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="22" customHeight="1">
+    <row r="5" spans="1:2" ht="22.05" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="8" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="A2:A5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"standard,discounted,out_of_stock,membership,multipack"</formula1>
@@ -481,6 +475,9 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{9DDCE113-522F-DC43-8D2E-243D7DAD9FC5}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{640083E5-C620-2845-AF78-E399B1AA87F6}"/>
     <hyperlink ref="B6" r:id="rId3" xr:uid="{84C2D311-926A-034E-8173-14C9775C0D7E}"/>
+    <hyperlink ref="B4" r:id="rId4" xr:uid="{C7FB0D21-D223-4E56-9248-9C035F8768BC}"/>
+    <hyperlink ref="B5" r:id="rId5" xr:uid="{E813C7C7-AB14-46E5-8BE0-164C200DFAB6}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{5B2A8AC4-9726-4650-B39E-47CB4A865DF0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
delete the unit, and unit price
</commit_message>
<xml_diff>
--- a/src/scraping/data/cold_start/tesco.xlsx
+++ b/src/scraping/data/cold_start/tesco.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yuding.Duan\OneDrive - Ipsos\3. self_projects\competitor_product_search\src\scraping\data\cold_start\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kumo/programming/competitor_product_search/src/scraping/data/cold_start/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74201E26-B69A-4231-98C0-B07962014AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BED166-91CB-534F-AA72-4A5D501C5588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5960" yWindow="760" windowWidth="24280" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cold_start" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>page_type</t>
   </si>
@@ -38,35 +38,45 @@
   </si>
   <si>
     <t>https://www.tesco.com/groceries/en-GB/products/276797313</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/325502056</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/305728358</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.tesco.com/shop/en-GB/products/330702828</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>discounted</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/322999875</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/330702828</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>discounted</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>https://www.tesco.com/shop/en-GB/products/330671337</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.tesco.com/shop/en-GB/products/287134166</t>
+  </si>
+  <si>
+    <t>membership</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.tesco.com/shop/en-GB/products/311961072</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -80,6 +90,10 @@
     <font>
       <sz val="11"/>
       <color rgb="FF1F2937"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Carlito"/>
     </font>
     <font>
@@ -172,26 +186,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="3">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -401,14 +418,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="22.05" customHeight="1">
+    <row r="1" spans="1:2" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -416,7 +433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="22.05" customHeight="1">
+    <row r="2" spans="1:2" ht="22" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -424,7 +441,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="22.05" customHeight="1">
+    <row r="3" spans="1:2" ht="22" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
@@ -432,40 +449,48 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="22.05" customHeight="1">
+    <row r="4" spans="1:2" ht="22" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="22.05" customHeight="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="22" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>11</v>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="A2:A5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"standard,discounted,out_of_stock,membership,multipack"</formula1>
@@ -475,9 +500,9 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{9DDCE113-522F-DC43-8D2E-243D7DAD9FC5}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{640083E5-C620-2845-AF78-E399B1AA87F6}"/>
     <hyperlink ref="B6" r:id="rId3" xr:uid="{84C2D311-926A-034E-8173-14C9775C0D7E}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{C7FB0D21-D223-4E56-9248-9C035F8768BC}"/>
-    <hyperlink ref="B5" r:id="rId5" xr:uid="{E813C7C7-AB14-46E5-8BE0-164C200DFAB6}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{5B2A8AC4-9726-4650-B39E-47CB4A865DF0}"/>
+    <hyperlink ref="B4" r:id="rId4" xr:uid="{77731F84-4284-CA4F-B358-F246F4DC3D93}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{6709BB5F-9053-B74F-89E3-5E061B30B32A}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{C09CA85A-D27F-9F43-BCC5-506676103E5F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
1. add page type availability 2. fix the scraper attention issue
</commit_message>
<xml_diff>
--- a/src/scraping/data/cold_start/tesco.xlsx
+++ b/src/scraping/data/cold_start/tesco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kumo/programming/competitor_product_search/src/scraping/data/cold_start/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BED166-91CB-534F-AA72-4A5D501C5588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5367D9-A987-8345-A221-AB3822F63DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5960" yWindow="760" windowWidth="24280" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,14 +61,15 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
+    <t>membership</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.tesco.com/shop/en-GB/products/311961072</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
     <t>https://www.tesco.com/shop/en-GB/products/287134166</t>
-  </si>
-  <si>
-    <t>membership</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/311961072</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -462,7 +463,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -483,10 +484,10 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -503,6 +504,7 @@
     <hyperlink ref="B4" r:id="rId4" xr:uid="{77731F84-4284-CA4F-B358-F246F4DC3D93}"/>
     <hyperlink ref="B7" r:id="rId5" xr:uid="{6709BB5F-9053-B74F-89E3-5E061B30B32A}"/>
     <hyperlink ref="B8" r:id="rId6" xr:uid="{C09CA85A-D27F-9F43-BCC5-506676103E5F}"/>
+    <hyperlink ref="B5" r:id="rId7" xr:uid="{C86FF34D-9C1B-4B41-B638-518C00C83F6F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>